<commit_message>
adding custom fields properly
</commit_message>
<xml_diff>
--- a/api/templates/device_activity/en.xlsx
+++ b/api/templates/device_activity/en.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\ubuntu\aspect\api\templates\device_activity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DB8EBB-19A3-43D6-9CC6-2C1D45B33839}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C18E7F8-194A-46F3-B2EC-243F5AD07222}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3669" yWindow="3669" windowWidth="24685" windowHeight="13148" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Errors by Device" sheetId="1" r:id="rId1"/>
+    <sheet name="Activity" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" fullPrecision="0"/>
 </workbook>

</xml_diff>

<commit_message>
Updating the status of the device
</commit_message>
<xml_diff>
--- a/api/templates/device_activity/en.xlsx
+++ b/api/templates/device_activity/en.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\ubuntu\aspect\api\templates\device_activity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C18E7F8-194A-46F3-B2EC-243F5AD07222}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAFA437-3894-41BA-AFF4-BFE60A5439DD}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3669" yWindow="3669" windowWidth="24685" windowHeight="13148" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activity" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullPrecision="0"/>
+  <calcPr calcId="181029" fullPrecision="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
@@ -59,6 +59,18 @@
   </si>
   <si>
     <t>Device Activity</t>
+  </si>
+  <si>
+    <t>Maintenance status</t>
+  </si>
+  <si>
+    <t>&lt;deviceApprovalStatus&gt;</t>
+  </si>
+  <si>
+    <t>&lt;deviceMaintenanceStatus&gt;</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -586,56 +598,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
     <col min="2" max="2" width="26.35546875" customWidth="1"/>
     <col min="3" max="3" width="18.140625" customWidth="1"/>
-    <col min="4" max="4" width="16.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29.5" style="2" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="16.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:6" ht="20.6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:4" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:6" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:4" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
@@ -645,11 +659,17 @@
       <c r="C7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
@@ -659,7 +679,13 @@
       <c r="C8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove total results column temporarily
</commit_message>
<xml_diff>
--- a/api/templates/device_activity/en.xlsx
+++ b/api/templates/device_activity/en.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-20.04\home\ubuntu\aspect\api\templates\device_activity\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\stefan\aspect\api\templates\device_activity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BAFA437-3894-41BA-AFF4-BFE60A5439DD}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB64437-6E89-40AA-9ACC-9CB9092CFB3E}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35571" yWindow="1329" windowWidth="22989" windowHeight="16080" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activity" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Last Upload</t>
   </si>
   <si>
-    <t>Total Tests Run During Period</t>
-  </si>
-  <si>
     <t>LGA: &lt;Lgas&gt;</t>
   </si>
   <si>
@@ -53,9 +50,6 @@
   </si>
   <si>
     <t>&lt;lastUploadOn&gt;</t>
-  </si>
-  <si>
-    <t>&lt;totalResults&gt;</t>
   </si>
   <si>
     <t>Device Activity</t>
@@ -201,22 +195,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -598,95 +583,88 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
     <col min="2" max="2" width="26.35546875" customWidth="1"/>
     <col min="3" max="3" width="18.140625" customWidth="1"/>
-    <col min="4" max="4" width="29.5" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="16.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="29.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="20.6" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" ht="20.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="2"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:6" ht="16.3" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:6" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A8" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed date formats and locked headers in templates
</commit_message>
<xml_diff>
--- a/api/templates/device_activity/en.xlsx
+++ b/api/templates/device_activity/en.xlsx
@@ -5,19 +5,30 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\device_activity\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\device_activity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51CD95E7-2D05-4AA0-934A-1EFF3847114B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4FCF52-F79D-4166-BA12-32FC2531CBEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activity Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Detailed by assay" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -95,8 +106,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -163,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -171,6 +183,8 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,47 +568,47 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.796875" customWidth="1"/>
-    <col min="2" max="2" width="26.296875" customWidth="1"/>
-    <col min="3" max="3" width="18.19921875" customWidth="1"/>
+    <col min="1" max="1" width="31.75" customWidth="1"/>
+    <col min="2" max="2" width="26.25" customWidth="1"/>
+    <col min="3" max="3" width="18.25" customWidth="1"/>
     <col min="4" max="4" width="29.5" customWidth="1"/>
-    <col min="5" max="5" width="18.796875" customWidth="1"/>
+    <col min="5" max="5" width="18.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -611,14 +625,14 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="4" t="s">
@@ -636,44 +650,44 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F113"/>
+  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="38.796875" customWidth="1"/>
-    <col min="3" max="3" width="37.296875" customWidth="1"/>
-    <col min="4" max="4" width="36.59765625" customWidth="1"/>
-    <col min="5" max="5" width="19.296875" customWidth="1"/>
-    <col min="6" max="6" width="17.19921875" customWidth="1"/>
+    <col min="1" max="2" width="38.75" customWidth="1"/>
+    <col min="3" max="3" width="37.25" customWidth="1"/>
+    <col min="4" max="4" width="36.625" customWidth="1"/>
+    <col min="5" max="5" width="19.25" customWidth="1"/>
+    <col min="6" max="6" width="17.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -693,7 +707,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -703,7 +717,7 @@
       <c r="C8" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="6" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="4" t="s">
@@ -713,8 +727,323 @@
         <v>14</v>
       </c>
     </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D9" s="6"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D11" s="6"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D12" s="6"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D13" s="6"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D14" s="6"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D16" s="6"/>
+    </row>
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D17" s="6"/>
+    </row>
+    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="6"/>
+    </row>
+    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D19" s="6"/>
+    </row>
+    <row r="20" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D20" s="6"/>
+    </row>
+    <row r="21" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D21" s="6"/>
+    </row>
+    <row r="22" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D22" s="6"/>
+    </row>
+    <row r="23" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D23" s="6"/>
+    </row>
+    <row r="24" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D24" s="6"/>
+    </row>
+    <row r="25" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D25" s="6"/>
+    </row>
+    <row r="26" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D26" s="6"/>
+    </row>
+    <row r="27" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D27" s="6"/>
+    </row>
+    <row r="28" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D28" s="6"/>
+    </row>
+    <row r="29" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D29" s="6"/>
+    </row>
+    <row r="30" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D30" s="6"/>
+    </row>
+    <row r="31" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D31" s="6"/>
+    </row>
+    <row r="32" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D32" s="6"/>
+    </row>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D33" s="6"/>
+    </row>
+    <row r="34" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D34" s="6"/>
+    </row>
+    <row r="35" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D35" s="6"/>
+    </row>
+    <row r="36" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D36" s="6"/>
+    </row>
+    <row r="37" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D37" s="6"/>
+    </row>
+    <row r="38" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D38" s="6"/>
+    </row>
+    <row r="39" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D39" s="6"/>
+    </row>
+    <row r="40" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D40" s="6"/>
+    </row>
+    <row r="41" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D41" s="6"/>
+    </row>
+    <row r="42" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D42" s="6"/>
+    </row>
+    <row r="43" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D43" s="6"/>
+    </row>
+    <row r="44" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D44" s="6"/>
+    </row>
+    <row r="45" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D45" s="6"/>
+    </row>
+    <row r="46" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D46" s="6"/>
+    </row>
+    <row r="47" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D47" s="6"/>
+    </row>
+    <row r="48" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D48" s="6"/>
+    </row>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D49" s="6"/>
+    </row>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D50" s="6"/>
+    </row>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D51" s="6"/>
+    </row>
+    <row r="52" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D52" s="6"/>
+    </row>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D53" s="6"/>
+    </row>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D54" s="6"/>
+    </row>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D55" s="6"/>
+    </row>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D56" s="6"/>
+    </row>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D57" s="6"/>
+    </row>
+    <row r="58" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D58" s="6"/>
+    </row>
+    <row r="59" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D59" s="6"/>
+    </row>
+    <row r="60" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D60" s="6"/>
+    </row>
+    <row r="61" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D61" s="6"/>
+    </row>
+    <row r="62" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D62" s="6"/>
+    </row>
+    <row r="63" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D63" s="6"/>
+    </row>
+    <row r="64" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D64" s="6"/>
+    </row>
+    <row r="65" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D65" s="6"/>
+    </row>
+    <row r="66" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D66" s="6"/>
+    </row>
+    <row r="67" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D67" s="6"/>
+    </row>
+    <row r="68" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D68" s="6"/>
+    </row>
+    <row r="69" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D69" s="6"/>
+    </row>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D70" s="6"/>
+    </row>
+    <row r="71" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D71" s="6"/>
+    </row>
+    <row r="72" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D72" s="6"/>
+    </row>
+    <row r="73" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D73" s="6"/>
+    </row>
+    <row r="74" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D74" s="6"/>
+    </row>
+    <row r="75" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D75" s="6"/>
+    </row>
+    <row r="76" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D76" s="6"/>
+    </row>
+    <row r="77" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D77" s="6"/>
+    </row>
+    <row r="78" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D78" s="6"/>
+    </row>
+    <row r="79" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D79" s="6"/>
+    </row>
+    <row r="80" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D80" s="6"/>
+    </row>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D81" s="6"/>
+    </row>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D82" s="6"/>
+    </row>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D83" s="6"/>
+    </row>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D84" s="6"/>
+    </row>
+    <row r="85" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D85" s="6"/>
+    </row>
+    <row r="86" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D86" s="6"/>
+    </row>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D87" s="6"/>
+    </row>
+    <row r="88" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D88" s="6"/>
+    </row>
+    <row r="89" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D89" s="6"/>
+    </row>
+    <row r="90" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D90" s="6"/>
+    </row>
+    <row r="91" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D91" s="6"/>
+    </row>
+    <row r="92" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D92" s="6"/>
+    </row>
+    <row r="93" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D93" s="6"/>
+    </row>
+    <row r="94" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D94" s="6"/>
+    </row>
+    <row r="95" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D95" s="6"/>
+    </row>
+    <row r="96" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D96" s="6"/>
+    </row>
+    <row r="97" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D97" s="6"/>
+    </row>
+    <row r="98" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D98" s="6"/>
+    </row>
+    <row r="99" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D99" s="6"/>
+    </row>
+    <row r="100" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D100" s="6"/>
+    </row>
+    <row r="101" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D101" s="6"/>
+    </row>
+    <row r="102" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D102" s="6"/>
+    </row>
+    <row r="103" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D103" s="6"/>
+    </row>
+    <row r="104" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D104" s="6"/>
+    </row>
+    <row r="105" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D105" s="6"/>
+    </row>
+    <row r="106" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D106" s="6"/>
+    </row>
+    <row r="107" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D107" s="6"/>
+    </row>
+    <row r="108" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D108" s="6"/>
+    </row>
+    <row r="109" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D109" s="6"/>
+    </row>
+    <row r="110" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D110" s="6"/>
+    </row>
+    <row r="111" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D111" s="6"/>
+    </row>
+    <row r="112" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D112" s="6"/>
+    </row>
+    <row r="113" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D113" s="6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>